<commit_message>
feat(config): ItemConfig 价格列与 initialCredits 配置、金币格式串导出；docs 回填 P1-M1 验收与 P1-M2 记录
- ItemConfig 四 sheet 增 sellPrice（全表=价值）/buyPrice（消耗品与 I/II 档装备=价值×2，其余 0，83 件中 21 件可购买）
- GlobalConfig 增 initialCredits=1000（服务端注册发放依据）；FormatText 的 LobbyCurrencyPending 改为 CREDITS: {0:N0} 格式串
- luban_export 重导 Gen 与 DataTables，同步服务端 config/
- TODO.md：P1-M1 人工验收回填、P1-M2 按服务端权威改写范围并记录实现；新增 .scratch/p1-m2/spec.md（决策/验证/人工验收清单）
</commit_message>
<xml_diff>
--- a/SBE-Design/Datas/FormatText_格式化文本.xlsx
+++ b/SBE-Design/Datas/FormatText_格式化文本.xlsx
@@ -1387,6 +1387,8 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
+    <row r="16"/>
     <row r="17" s="17">
       <c r="B17" s="15" t="inlineStr">
         <is>
@@ -1399,6 +1401,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" s="17">
       <c r="B19" s="15" t="inlineStr">
         <is>
@@ -1694,7 +1697,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>CREDITS: —</t>
+          <t>CREDITS: {0:N0}</t>
         </is>
       </c>
     </row>

</xml_diff>